<commit_message>
Add missing variables to template
</commit_message>
<xml_diff>
--- a/settlement/Inequality Input Data Template CMCC Settlement EMPTY.xlsx
+++ b/settlement/Inequality Input Data Template CMCC Settlement EMPTY.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emmerling\CMCC Dropbox\Johannes Emmerling\EIEE\NAVIGATE\NAVIGATE-RESEARCH\WP4 Inequality\inequality-dataset-for-iams\settlement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D522F1C-B82F-455C-91BD-FC9C0E1373F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7844487-D14E-43C9-98F3-D93AE23E67FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7B1F585D-5655-48D5-9EC0-02F8EFD3D86B}"/>
   </bookViews>
   <sheets>
     <sheet name="Inequality Input Data Template " sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="77">
   <si>
     <t>MODEL</t>
   </si>
@@ -239,13 +252,25 @@
   </si>
   <si>
     <t>Digital Access|Electric Grid|Rural|Dx</t>
+  </si>
+  <si>
+    <t>Expenditure Share|Urban</t>
+  </si>
+  <si>
+    <t>Share of TOTAL Expenditures of Urban Households</t>
+  </si>
+  <si>
+    <t>Expenditure Share|Rural</t>
+  </si>
+  <si>
+    <t>Share of TOTAL Expenditures of Rural Households</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,6 +401,13 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -722,8 +754,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1099,8 +1132,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DA951D2-50BA-4D44-A188-00AF4DB0B195}">
-  <dimension ref="A1:AO51"/>
+  <dimension ref="A1:AO53"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="36.90625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1283,18 +1319,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:41" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
-        <v>17</v>
+    <row r="6" spans="1:41" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:41" x14ac:dyDescent="0.35">
@@ -1302,7 +1338,7 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
@@ -1316,7 +1352,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
         <v>8</v>
@@ -1327,10 +1363,10 @@
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
         <v>8</v>
@@ -1341,10 +1377,10 @@
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
         <v>8</v>
@@ -1355,24 +1391,24 @@
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
@@ -1386,7 +1422,7 @@
         <v>6</v>
       </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
@@ -1400,7 +1436,7 @@
         <v>6</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" t="s">
         <v>8</v>
@@ -1414,7 +1450,7 @@
         <v>6</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E15" t="s">
         <v>8</v>
@@ -1428,10 +1464,13 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
@@ -1439,24 +1478,21 @@
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
@@ -1464,13 +1500,13 @@
         <v>20</v>
       </c>
       <c r="D19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E19" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="F19" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
@@ -1478,13 +1514,13 @@
         <v>20</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E20" t="s">
         <v>36</v>
       </c>
       <c r="F20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
@@ -1492,27 +1528,27 @@
         <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E21" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="F21" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E22" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="F22" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
@@ -1520,13 +1556,13 @@
         <v>6</v>
       </c>
       <c r="D23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E23" t="s">
         <v>8</v>
       </c>
       <c r="F23" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
@@ -1534,13 +1570,13 @@
         <v>6</v>
       </c>
       <c r="D24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E24" t="s">
         <v>8</v>
       </c>
       <c r="F24" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
@@ -1548,13 +1584,13 @@
         <v>6</v>
       </c>
       <c r="D25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E25" t="s">
         <v>8</v>
       </c>
       <c r="F25" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
@@ -1562,27 +1598,27 @@
         <v>6</v>
       </c>
       <c r="D26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E26" t="s">
         <v>8</v>
       </c>
       <c r="F26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" t="s">
-        <v>48</v>
-      </c>
-      <c r="E27" t="s">
-        <v>8</v>
-      </c>
-      <c r="F27" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
@@ -1590,7 +1626,7 @@
         <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E28" t="s">
         <v>8</v>
@@ -1601,10 +1637,10 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D29" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E29" t="s">
         <v>8</v>
@@ -1618,7 +1654,7 @@
         <v>6</v>
       </c>
       <c r="D30" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E30" t="s">
         <v>8</v>
@@ -1632,13 +1668,13 @@
         <v>20</v>
       </c>
       <c r="D31" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E31" t="s">
         <v>8</v>
       </c>
       <c r="F31" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
@@ -1646,21 +1682,21 @@
         <v>6</v>
       </c>
       <c r="D32" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E32" t="s">
         <v>8</v>
       </c>
       <c r="F32" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E33" t="s">
         <v>8</v>
@@ -1674,7 +1710,7 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E34" t="s">
         <v>8</v>
@@ -1688,7 +1724,7 @@
         <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E35" t="s">
         <v>8</v>
@@ -1702,10 +1738,13 @@
         <v>6</v>
       </c>
       <c r="D36" t="s">
-        <v>57</v>
+        <v>55</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
       </c>
       <c r="F36" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
@@ -1713,38 +1752,35 @@
         <v>6</v>
       </c>
       <c r="D37" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
       </c>
       <c r="F37" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D38" t="s">
-        <v>59</v>
-      </c>
-      <c r="E38" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="F38" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E39" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="F39" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
@@ -1752,13 +1788,13 @@
         <v>20</v>
       </c>
       <c r="D40" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E40" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="F40" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
@@ -1766,70 +1802,82 @@
         <v>20</v>
       </c>
       <c r="D41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E41" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="F41" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D42" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E42" t="s">
-        <v>8</v>
+        <v>36</v>
+      </c>
+      <c r="F42" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D43" t="s">
+        <v>62</v>
+      </c>
+      <c r="E43" t="s">
+        <v>41</v>
+      </c>
+      <c r="F43" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E43" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="E45" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" t="s">
         <v>65</v>
       </c>
-      <c r="E44" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="E46" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" t="s">
         <v>66</v>
-      </c>
-      <c r="E45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D46" t="s">
-        <v>67</v>
-      </c>
-      <c r="E46" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D47" t="s">
-        <v>68</v>
       </c>
       <c r="E47" t="s">
         <v>8</v>
@@ -1837,7 +1885,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="D48" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E48" t="s">
         <v>8</v>
@@ -1845,7 +1893,7 @@
     </row>
     <row r="49" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D49" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E49" t="s">
         <v>8</v>
@@ -1853,7 +1901,7 @@
     </row>
     <row r="50" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D50" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E50" t="s">
         <v>8</v>
@@ -1861,9 +1909,25 @@
     </row>
     <row r="51" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D51" t="s">
+        <v>70</v>
+      </c>
+      <c r="E51" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D52" t="s">
+        <v>71</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D53" t="s">
         <v>72</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E53" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>